<commit_message>
Índices: «11.130» se rechaza como ambiguo y la plantilla lee los números como la importación
«11.130» sin coma puede ser 11130 o 11,13: la importación lo leía como 11,13 y la
plantilla de Excel mostraba 11130. Además, la fórmula de la plantilla leía «8834.3» como
88343 y, como la lectura toma lo que calculó Excel, se importaba eso.

- El pegado y la plantilla rechazan el valor ambiguo con «"11.130" es ambiguo: escribilo
  11130 o 11.130,0». La importación de estructuras no cambia.
- Las fórmulas de los meses siguen la regla de la importación (sin coma, el punto es el
  decimal) y dejan vacío el valor ambiguo.
- La plantilla pasa a la versión 2: una de la versión 1 se rechaza para que se descargue
  de nuevo.
- Tests que evalúan las fórmulas con ClosedXML. La planilla guardada con Excel real se
  rehízo en la versión 2 y la anterior queda para el test del rechazo.
</commit_message>
<xml_diff>
--- a/tests/SIGO.Tests/Datos/plantilla-indices-guardada-en-excel.xlsx
+++ b/tests/SIGO.Tests/Datos/plantilla-indices-guardada-en-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ncarracedo\Documents\sigotest-source\artifacts\plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ncarracedo\Documents\sigotest-source\artifacts\auditoria\p3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD68534C-6DD0-4B8D-811E-1730163FF45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C41F215-913A-41D4-AF54-AED715827BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="164">
   <si>
     <t>ID publicación</t>
   </si>
@@ -246,12 +246,6 @@
     <t>k</t>
   </si>
   <si>
-    <t>COSTO_FINANCIERO</t>
-  </si>
-  <si>
-    <t>Costo Financiero – Tasas Activas Banco Nación</t>
-  </si>
-  <si>
     <t>ELECTROBOMBA</t>
   </si>
   <si>
@@ -522,16 +516,16 @@
     <t>9.586,3  9.796,6  9.974,6  10.287,4  10.420,6  10.820,1  10.976,4  11.318,9  11.542,6  11.819,6  12.319,1  12.724,8  13.074,3</t>
   </si>
   <si>
+    <t>12.804,4	13.848,9 14.136,0 s 15.884,0  15.690,8  16.241,4  16.278,9  15.696,1  15.869,9  14.655,4  14.985,6  15.654,6</t>
+  </si>
+  <si>
+    <t>12.746,9  12.801,0  13.030,3</t>
+  </si>
+  <si>
+    <t>15.007,6</t>
+  </si>
+  <si>
     <t>Mano de obra (Cuadro 1.4) 100,0 8.943,3  9.143,5  9.295,7  9.591,7  9.715,6  10.118,9  10.260,4  10.618,6  10.826,9  11.061,1  11.603,5  12.006,6  12.401,3</t>
-  </si>
-  <si>
-    <t>12.804,4	13.848,9 14.136,0 s 15.884,0  15.690,8  16.241,4  16.278,9  15.696,1  15.869,9  14.655,4  14.985,6  15.654,6</t>
-  </si>
-  <si>
-    <t>12.746,9  12.801,0  13.030,3</t>
-  </si>
-  <si>
-    <t>15.007,6</t>
   </si>
 </sst>
 </file>
@@ -920,7 +914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U44"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -944,7 +938,7 @@
         <v>2</v>
       </c>
       <c r="E1">
-        <f>COUNT(G5:S44)</f>
+        <f>COUNT(G5:S43)</f>
         <v>42</v>
       </c>
     </row>
@@ -1040,65 +1034,65 @@
         <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G5" s="6">
-        <f t="shared" ref="G5:G44" si="0">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)),",",".")),"")</f>
+        <f t="shared" ref="G5:G43" si="0">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1,300)),".",",")))),"")</f>
         <v>9586.2999999999993</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" ref="H5:H44" si="1">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)),",",".")),"")</f>
+        <f t="shared" ref="H5:H43" si="1">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),301,300)),".",",")))),"")</f>
         <v>9796.6</v>
       </c>
       <c r="I5" s="6">
-        <f t="shared" ref="I5:I44" si="2">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)),",",".")),"")</f>
+        <f t="shared" ref="I5:I43" si="2">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),601,300)),".",",")))),"")</f>
         <v>9974.6</v>
       </c>
       <c r="J5" s="6">
-        <f t="shared" ref="J5:J44" si="3">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)),",",".")),"")</f>
+        <f t="shared" ref="J5:J43" si="3">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),901,300)),".",",")))),"")</f>
         <v>10287.4</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" ref="K5:K44" si="4">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)),",",".")),"")</f>
+        <f t="shared" ref="K5:K43" si="4">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1201,300)),".",",")))),"")</f>
         <v>10420.6</v>
       </c>
       <c r="L5" s="6">
-        <f t="shared" ref="L5:L44" si="5">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)),",",".")),"")</f>
+        <f t="shared" ref="L5:L43" si="5">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1501,300)),".",",")))),"")</f>
         <v>10820.1</v>
       </c>
       <c r="M5" s="6">
-        <f t="shared" ref="M5:M44" si="6">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)),",",".")),"")</f>
+        <f t="shared" ref="M5:M43" si="6">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),1801,300)),".",",")))),"")</f>
         <v>10976.4</v>
       </c>
       <c r="N5" s="6">
-        <f t="shared" ref="N5:N44" si="7">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)),",",".")),"")</f>
+        <f t="shared" ref="N5:N43" si="7">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2101,300)),".",",")))),"")</f>
         <v>11318.9</v>
       </c>
       <c r="O5" s="6">
-        <f t="shared" ref="O5:O44" si="8">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)),",",".")),"")</f>
+        <f t="shared" ref="O5:O43" si="8">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2401,300)),".",",")))),"")</f>
         <v>11542.6</v>
       </c>
       <c r="P5" s="6">
-        <f t="shared" ref="P5:P44" si="9">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)),",",".")),"")</f>
+        <f t="shared" ref="P5:P43" si="9">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),2701,300)),".",",")))),"")</f>
         <v>11819.6</v>
       </c>
       <c r="Q5" s="6">
-        <f t="shared" ref="Q5:Q44" si="10">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)),",",".")),"")</f>
+        <f t="shared" ref="Q5:Q43" si="10">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3001,300)),".",",")))),"")</f>
         <v>12319.1</v>
       </c>
       <c r="R5" s="6">
-        <f t="shared" ref="R5:R44" si="11">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)),",",".")),"")</f>
+        <f t="shared" ref="R5:R43" si="11">IFERROR(IF(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U5," ",REPT(" ",300)),3301,300)),".",",")))),"")</f>
         <v>12724.8</v>
       </c>
       <c r="S5" s="6">
         <v>13100</v>
       </c>
       <c r="T5" t="str">
-        <f t="shared" ref="T5:T44" si="12">TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5,CHAR(9)," "),CHAR(160)," "),CHAR(10)," "),CHAR(13)," "))</f>
+        <f t="shared" ref="T5:T43" si="12">TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F5,CHAR(9)," "),CHAR(160)," "),CHAR(10)," "),CHAR(13)," "))</f>
         <v>9.586,3 9.796,6 9.974,6 10.287,4 10.420,6 10.820,1 10.976,4 11.318,9 11.542,6 11.819,6 12.319,1 12.724,8 13.074,3</v>
       </c>
       <c r="U5" t="str">
-        <f t="shared" ref="U5:U44" si="13">IF(ISNUMBER(SEARCH(" 100,0 "," "&amp;T5&amp;" ")),TRIM(MID(" "&amp;T5&amp;" ",SEARCH(" 100,0 "," "&amp;T5&amp;" ")+7,9999)),T5)</f>
+        <f t="shared" ref="U5:U43" si="13">IF(ISNUMBER(SEARCH(" 100,0 "," "&amp;T5&amp;" ")),TRIM(MID(" "&amp;T5&amp;" ",SEARCH(" 100,0 "," "&amp;T5&amp;" ")+7,9999)),T5)</f>
         <v>9.586,3 9.796,6 9.974,6 10.287,4 10.420,6 10.820,1 10.976,4 11.318,9 11.542,6 11.819,6 12.319,1 12.724,8 13.074,3</v>
       </c>
     </row>
@@ -1168,7 +1162,7 @@
         <v/>
       </c>
       <c r="S6" s="6" t="str">
-        <f t="shared" ref="S5:S44" si="14">IFERROR(IF(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300))="","",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)),",",".")),"")</f>
+        <f t="shared" ref="S5:S43" si="14">IFERROR(IF(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300))="","",IF(ISNUMBER(FIND(",",TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)))),_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)),",","."),IF(AND(LEN(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)))-LEN(SUBSTITUTE(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)),".",""))=1,LEN(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)))-FIND(".",TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300))&amp;".")=3,FIND(".",TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300))&amp;".")&lt;=4,ISNUMBER(-LEFT(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)),1))),"",_xlfn.NUMBERVALUE(TRIM(MID(SUBSTITUTE($U6," ",REPT(" ",300)),3601,300)),".",",")))),"")</f>
         <v/>
       </c>
       <c r="T6" t="str">
@@ -1587,7 +1581,7 @@
         <v>42</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
@@ -1745,7 +1739,7 @@
         <v>50</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
@@ -1903,7 +1897,7 @@
         <v>20</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
@@ -2208,13 +2202,13 @@
         <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="D20" t="s">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="6" t="str">
@@ -2280,19 +2274,19 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E21" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="6" t="str">
@@ -2358,19 +2352,19 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="6" t="str">
@@ -2436,16 +2430,16 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E23" t="s">
         <v>20</v>
@@ -2514,19 +2508,19 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="D24" t="s">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="F24" s="5"/>
       <c r="G24" s="6" t="str">
@@ -2592,19 +2586,19 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="6" t="str">
@@ -2670,19 +2664,19 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>93</v>
+        <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="6" t="str">
@@ -2748,19 +2742,19 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="6" t="str">
@@ -2826,19 +2820,19 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="6" t="str">
@@ -2904,19 +2898,19 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="D29" t="s">
-        <v>16</v>
+        <v>106</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="6" t="str">
@@ -2982,16 +2976,16 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B30" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C30" t="s">
         <v>20</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E30" t="s">
         <v>20</v>
@@ -3060,16 +3054,16 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C31" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="D31" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="E31" t="s">
         <v>20</v>
@@ -3138,177 +3132,177 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32" s="5"/>
-      <c r="G32" s="6" t="str">
+        <v>116</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="G32" s="6">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H32" s="6" t="str">
+        <v>8943.2999999999993</v>
+      </c>
+      <c r="H32" s="6">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I32" s="6" t="str">
+        <v>9143.5</v>
+      </c>
+      <c r="I32" s="6">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J32" s="6" t="str">
+        <v>9295.7000000000007</v>
+      </c>
+      <c r="J32" s="6">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K32" s="6" t="str">
+        <v>9591.7000000000007</v>
+      </c>
+      <c r="K32" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L32" s="6" t="str">
+        <v>9715.6</v>
+      </c>
+      <c r="L32" s="6">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M32" s="6" t="str">
+        <v>10118.9</v>
+      </c>
+      <c r="M32" s="6">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N32" s="6" t="str">
+        <v>10260.4</v>
+      </c>
+      <c r="N32" s="6">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="O32" s="6" t="str">
+        <v>10618.6</v>
+      </c>
+      <c r="O32" s="6">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="P32" s="6" t="str">
+        <v>10826.9</v>
+      </c>
+      <c r="P32" s="6">
         <f t="shared" si="9"/>
-        <v/>
-      </c>
-      <c r="Q32" s="6" t="str">
+        <v>11061.1</v>
+      </c>
+      <c r="Q32" s="6">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="R32" s="6" t="str">
+        <v>11603.5</v>
+      </c>
+      <c r="R32" s="6">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="S32" s="6" t="str">
+        <v>12006.6</v>
+      </c>
+      <c r="S32" s="6">
         <f t="shared" si="14"/>
-        <v/>
+        <v>12401.3</v>
       </c>
       <c r="T32" t="str">
         <f t="shared" si="12"/>
-        <v/>
+        <v>Mano de obra (Cuadro 1.4) 100,0 8.943,3 9.143,5 9.295,7 9.591,7 9.715,6 10.118,9 10.260,4 10.618,6 10.826,9 11.061,1 11.603,5 12.006,6 12.401,3</v>
       </c>
       <c r="U32" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v>8.943,3 9.143,5 9.295,7 9.591,7 9.715,6 10.118,9 10.260,4 10.618,6 10.826,9 11.061,1 11.603,5 12.006,6 12.401,3</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C33" t="s">
-        <v>117</v>
+        <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="E33" t="s">
-        <v>118</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="G33" s="6">
+        <v>20</v>
+      </c>
+      <c r="F33" s="5"/>
+      <c r="G33" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>8943.2999999999993</v>
-      </c>
-      <c r="H33" s="6">
+        <v/>
+      </c>
+      <c r="H33" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>9143.5</v>
-      </c>
-      <c r="I33" s="6">
+        <v/>
+      </c>
+      <c r="I33" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>9295.7000000000007</v>
-      </c>
-      <c r="J33" s="6">
+        <v/>
+      </c>
+      <c r="J33" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>9591.7000000000007</v>
-      </c>
-      <c r="K33" s="6">
+        <v/>
+      </c>
+      <c r="K33" s="6" t="str">
         <f t="shared" si="4"/>
-        <v>9715.6</v>
-      </c>
-      <c r="L33" s="6">
+        <v/>
+      </c>
+      <c r="L33" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>10118.9</v>
-      </c>
-      <c r="M33" s="6">
+        <v/>
+      </c>
+      <c r="M33" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>10260.4</v>
-      </c>
-      <c r="N33" s="6">
+        <v/>
+      </c>
+      <c r="N33" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>10618.6</v>
-      </c>
-      <c r="O33" s="6">
+        <v/>
+      </c>
+      <c r="O33" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>10826.9</v>
-      </c>
-      <c r="P33" s="6">
+        <v/>
+      </c>
+      <c r="P33" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>11061.1</v>
-      </c>
-      <c r="Q33" s="6">
+        <v/>
+      </c>
+      <c r="Q33" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>11603.5</v>
-      </c>
-      <c r="R33" s="6">
+        <v/>
+      </c>
+      <c r="R33" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>12006.6</v>
-      </c>
-      <c r="S33" s="6">
+        <v/>
+      </c>
+      <c r="S33" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>12401.3</v>
+        <v/>
       </c>
       <c r="T33" t="str">
         <f t="shared" si="12"/>
-        <v>Mano de obra (Cuadro 1.4) 100,0 8.943,3 9.143,5 9.295,7 9.591,7 9.715,6 10.118,9 10.260,4 10.618,6 10.826,9 11.061,1 11.603,5 12.006,6 12.401,3</v>
+        <v/>
       </c>
       <c r="U33" t="str">
         <f t="shared" si="13"/>
-        <v>8.943,3 9.143,5 9.295,7 9.591,7 9.715,6 10.118,9 10.260,4 10.618,6 10.826,9 11.061,1 11.603,5 12.006,6 12.401,3</v>
+        <v/>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C34" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="D34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E34" t="s">
-        <v>20</v>
+        <v>124</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="6" t="str">
@@ -3374,19 +3368,19 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B35" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C35" t="s">
-        <v>124</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E35" t="s">
-        <v>126</v>
+        <v>20</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="6" t="str">
@@ -3452,19 +3446,19 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C36" t="s">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="D36" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E36" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="6" t="str">
@@ -3530,19 +3524,19 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F37" s="5"/>
       <c r="G37" s="6" t="str">
@@ -3608,19 +3602,19 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="D38" t="s">
-        <v>20</v>
+        <v>139</v>
       </c>
       <c r="E38" t="s">
-        <v>138</v>
+        <v>20</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="6" t="str">
@@ -3686,19 +3680,19 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>141</v>
+        <v>20</v>
       </c>
       <c r="E39" t="s">
-        <v>20</v>
+        <v>143</v>
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="6" t="str">
@@ -3764,19 +3758,19 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C40" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="D40" t="s">
-        <v>20</v>
+        <v>146</v>
       </c>
       <c r="E40" t="s">
-        <v>145</v>
+        <v>20</v>
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="6" t="str">
@@ -3842,19 +3836,19 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C41" t="s">
-        <v>20</v>
+        <v>149</v>
       </c>
       <c r="D41" t="s">
-        <v>148</v>
+        <v>20</v>
       </c>
       <c r="E41" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="F41" s="5"/>
       <c r="G41" s="6" t="str">
@@ -3920,19 +3914,19 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B42" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C42" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D42" t="s">
         <v>20</v>
       </c>
       <c r="E42" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F42" s="5"/>
       <c r="G42" s="6" t="str">
@@ -3998,19 +3992,19 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B43" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C43" t="s">
-        <v>155</v>
+        <v>20</v>
       </c>
       <c r="D43" t="s">
-        <v>20</v>
+        <v>157</v>
       </c>
       <c r="E43" t="s">
-        <v>156</v>
+        <v>20</v>
       </c>
       <c r="F43" s="5"/>
       <c r="G43" s="6" t="str">
@@ -4074,87 +4068,9 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>157</v>
-      </c>
-      <c r="B44" t="s">
-        <v>158</v>
-      </c>
-      <c r="C44" t="s">
-        <v>20</v>
-      </c>
-      <c r="D44" t="s">
-        <v>159</v>
-      </c>
-      <c r="E44" t="s">
-        <v>20</v>
-      </c>
-      <c r="F44" s="5"/>
-      <c r="G44" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H44" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I44" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J44" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K44" s="6" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="L44" s="6" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="M44" s="6" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="N44" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="O44" s="6" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="P44" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v/>
-      </c>
-      <c r="Q44" s="6" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="R44" s="6" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="S44" s="6" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="T44" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="U44" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="El valor de un mes tiene que ser un número mayor que cero." sqref="G5:S44" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="El valor de un mes tiene que ser un número mayor que cero." sqref="G5:S43" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4169,10 +4085,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>